<commit_message>
Prefill Chinese Leveling Forecast translations
</commit_message>
<xml_diff>
--- a/docs/localization/FafnyirTools_Leveling_Forecast_Chinese_Localization_Worksheet.xlsx
+++ b/docs/localization/FafnyirTools_Leveling_Forecast_Chinese_Localization_Worksheet.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R83b3810396ed4b81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strings" sheetId="2" r:id="R9c234e152a874b33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R17e4db8f350a4e86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strings" sheetId="2" r:id="Ra2a7963197e243f6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -222,7 +222,51 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="3">
+  <x:dxfs count="7">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF274E13"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFD9EAD3"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF073763"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCFE2F3"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF783F04"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE5CD"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF783F04"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFCE5CD"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
@@ -248,11 +292,11 @@
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FF783F04"/>
+        <x:color rgb="FF990000"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFCE5CD"/>
+          <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -505,7 +549,7 @@
         <x:v>Translator</x:v>
       </x:c>
       <x:c r="B4" s="13" t="str">
-        <x:v>Prepared for Yilang. Fill zhCN, zhTW, or both according to fluency in the matching World of Warcraft client.</x:v>
+        <x:v>A first-pass zhCN and zhTW translation is included. Yilang should review official World of Warcraft terminology, natural phrasing, and in-game fit.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
@@ -545,7 +589,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B9" s="13" t="str">
-        <x:v>Set Status to Translated when an entry is ready. A second fluent reviewer may set it to Reviewed after checking terminology and in-game context.</x:v>
+        <x:v>AI-drafted rows are marked Needs Review. Set Status to Translated after translator approval, or Reviewed after a second fluent review and contextual check.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -654,12 +698,16 @@
       <x:c r="F2" s="9" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="G2" s="26" t="str"/>
-      <x:c r="H2" s="26" t="str"/>
+      <x:c r="G2" s="26" t="str">
+        <x:v>升级预测</x:v>
+      </x:c>
+      <x:c r="H2" s="26" t="str">
+        <x:v>升級預測</x:v>
+      </x:c>
       <x:c r="I2" s="26" t="str"/>
       <x:c r="J2" s="25" t="str"/>
       <x:c r="K2" s="25" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Needs Review</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -681,12 +729,16 @@
       <x:c r="F3" s="9" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="G3" s="26" t="str"/>
-      <x:c r="H3" s="26" t="str"/>
+      <x:c r="G3" s="26" t="str">
+        <x:v>当前进度</x:v>
+      </x:c>
+      <x:c r="H3" s="26" t="str">
+        <x:v>目前進度</x:v>
+      </x:c>
       <x:c r="I3" s="26" t="str"/>
       <x:c r="J3" s="25" t="str"/>
       <x:c r="K3" s="25" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Needs Review</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -708,12 +760,16 @@
       <x:c r="F4" s="9" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="G4" s="26" t="str"/>
-      <x:c r="H4" s="26" t="str"/>
+      <x:c r="G4" s="26" t="str">
+        <x:v>已达最高等级</x:v>
+      </x:c>
+      <x:c r="H4" s="26" t="str">
+        <x:v>已達最高等級</x:v>
+      </x:c>
       <x:c r="I4" s="26" t="str"/>
       <x:c r="J4" s="25" t="str"/>
       <x:c r="K4" s="25" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Needs Review</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
@@ -735,14 +791,18 @@
       <x:c r="F5" s="9" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="G5" s="26" t="str"/>
-      <x:c r="H5" s="26" t="str"/>
+      <x:c r="G5" s="26" t="str">
+        <x:v>等级 %d — %s</x:v>
+      </x:c>
+      <x:c r="H5" s="26" t="str">
+        <x:v>等級 %d — %s</x:v>
+      </x:c>
       <x:c r="I5" s="26" t="str">
         <x:v>Preserve %d and %s.</x:v>
       </x:c>
       <x:c r="J5" s="25" t="str"/>
       <x:c r="K5" s="25" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Needs Review</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -764,12 +824,16 @@
       <x:c r="F6" s="9" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="G6" s="26" t="str"/>
-      <x:c r="H6" s="26" t="str"/>
+      <x:c r="G6" s="26" t="str">
+        <x:v>已完成且可交付的任务</x:v>
+      </x:c>
+      <x:c r="H6" s="26" t="str">
+        <x:v>已完成且可交付的任務</x:v>
+      </x:c>
       <x:c r="I6" s="26" t="str"/>
       <x:c r="J6" s="25" t="str"/>
       <x:c r="K6" s="25" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Needs Review</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -791,12 +855,16 @@
       <x:c r="F7" s="9" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="G7" s="26" t="str"/>
-      <x:c r="H7" s="26" t="str"/>
+      <x:c r="G7" s="26" t="str">
+        <x:v>已完成任务经验值</x:v>
+      </x:c>
+      <x:c r="H7" s="26" t="str">
+        <x:v>已完成任務經驗值</x:v>
+      </x:c>
       <x:c r="I7" s="26" t="str"/>
       <x:c r="J7" s="25" t="str"/>
       <x:c r="K7" s="25" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Needs Review</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -818,12 +886,16 @@
       <x:c r="F8" s="9" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="G8" s="26" t="str"/>
-      <x:c r="H8" s="26" t="str"/>
+      <x:c r="G8" s="26" t="str">
+        <x:v>有效任务经验加成</x:v>
+      </x:c>
+      <x:c r="H8" s="26" t="str">
+        <x:v>有效任務經驗加成</x:v>
+      </x:c>
       <x:c r="I8" s="26" t="str"/>
       <x:c r="J8" s="25" t="str"/>
       <x:c r="K8" s="25" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Needs Review</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -845,12 +917,16 @@
       <x:c r="F9" s="9" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="G9" s="26" t="str"/>
-      <x:c r="H9" s="26" t="str"/>
+      <x:c r="G9" s="26" t="str">
+        <x:v>不可用</x:v>
+      </x:c>
+      <x:c r="H9" s="26" t="str">
+        <x:v>無法取得</x:v>
+      </x:c>
       <x:c r="I9" s="26" t="str"/>
       <x:c r="J9" s="25" t="str"/>
       <x:c r="K9" s="25" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Needs Review</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -872,12 +948,16 @@
       <x:c r="F10" s="9" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="G10" s="26" t="str"/>
-      <x:c r="H10" s="26" t="str"/>
+      <x:c r="G10" s="26" t="str">
+        <x:v>交付任务后的预计进度</x:v>
+      </x:c>
+      <x:c r="H10" s="26" t="str">
+        <x:v>交付任務後的預估進度</x:v>
+      </x:c>
       <x:c r="I10" s="26" t="str"/>
       <x:c r="J10" s="25" t="str"/>
       <x:c r="K10" s="25" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Needs Review</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="24" hidden="0" customHeight="1">
@@ -899,14 +979,18 @@
       <x:c r="F11" s="9" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="G11" s="26" t="str"/>
-      <x:c r="H11" s="26" t="str"/>
+      <x:c r="G11" s="26" t="str">
+        <x:v>等级 %d+ — 超出下一级 %s 点经验值</x:v>
+      </x:c>
+      <x:c r="H11" s="26" t="str">
+        <x:v>等級 %d+ — 超出下一級 %s 點經驗值</x:v>
+      </x:c>
       <x:c r="I11" s="26" t="str">
         <x:v>Preserve %d, %s, and the + meaning.</x:v>
       </x:c>
       <x:c r="J11" s="25" t="str"/>
       <x:c r="K11" s="25" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Needs Review</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" hidden="0" customHeight="1">
@@ -928,14 +1012,18 @@
       <x:c r="F12" s="9" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="G12" s="26" t="str"/>
-      <x:c r="H12" s="26" t="str"/>
+      <x:c r="G12" s="26" t="str">
+        <x:v>使用暴雪调整后的任务经验值，包括适用的战团及其他加成。</x:v>
+      </x:c>
+      <x:c r="H12" s="26" t="str">
+        <x:v>使用暴雪調整後的任務經驗值，包括適用的戰隊及其他加成。</x:v>
+      </x:c>
       <x:c r="I12" s="26" t="str">
         <x:v>Keep Blizzard and Warband as official game terminology.</x:v>
       </x:c>
       <x:c r="J12" s="25" t="str"/>
       <x:c r="K12" s="25" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Needs Review</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -957,28 +1045,33 @@
       <x:c r="F13" s="9" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="G13" s="26" t="str"/>
-      <x:c r="H13" s="26" t="str"/>
+      <x:c r="G13" s="26" t="str">
+        <x:v>重新打开此页面以刷新。</x:v>
+      </x:c>
+      <x:c r="H13" s="26" t="str">
+        <x:v>重新開啟此頁面以更新。</x:v>
+      </x:c>
       <x:c r="I13" s="26" t="str"/>
       <x:c r="J13" s="25" t="str"/>
       <x:c r="K13" s="25" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Needs Review</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="K2:K13">
-    <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Translated"/>
-    <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Reviewed"/>
-    <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Needs Discussion"/>
+    <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Needs Review"/>
+    <x:cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="Translated"/>
+    <x:cfRule type="containsText" dxfId="5" priority="3" operator="containsText" text="Reviewed"/>
+    <x:cfRule type="containsText" dxfId="6" priority="4" operator="containsText" text="Needs Discussion"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="K2:K13">
-      <x:formula1>"Not Started,Translated,Reviewed,Needs Discussion"</x:formula1>
+      <x:formula1>"Not Started,Needs Review,Translated,Reviewed,Needs Discussion"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6064e4102e5422b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc2f74ae7dea4f08"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>